<commit_message>
System refresh - replacing repository with current local codebase
</commit_message>
<xml_diff>
--- a/details/C file -  register 19.03.2024..xlsx
+++ b/details/C file -  register 19.03.2024..xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\arosh\Downloads\CCU_CMA\details\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AROSHA\Downloads\CCU_CMA\details\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B6BBCB1-0543-40F7-8B5F-F70808AAF368}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A848CE52-7682-4293-8A41-53193634BAF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -7796,7 +7796,7 @@
     <t>Unauthorised Construction</t>
   </si>
   <si>
-    <t>Closed</t>
+    <t>Pending</t>
   </si>
 </sst>
 </file>
@@ -8660,19 +8660,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J639"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="37.5" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="37.5" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="11.109375" style="13" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.6640625" style="11" customWidth="1"/>
-    <col min="3" max="3" width="42.6640625" style="11" customWidth="1"/>
-    <col min="4" max="4" width="50.88671875" style="11" customWidth="1"/>
-    <col min="5" max="5" width="15.5546875" style="14" customWidth="1"/>
+    <col min="1" max="1" width="11.140625" style="13" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.7109375" style="11" customWidth="1"/>
+    <col min="3" max="3" width="42.7109375" style="11" customWidth="1"/>
+    <col min="4" max="4" width="50.85546875" style="11" customWidth="1"/>
+    <col min="5" max="5" width="15.5703125" style="14" customWidth="1"/>
     <col min="6" max="6" width="40" style="14" customWidth="1"/>
-    <col min="7" max="7" width="45.109375" style="11" customWidth="1"/>
-    <col min="8" max="8" width="36.33203125" style="15" customWidth="1"/>
-    <col min="9" max="9" width="13.44140625" style="13" customWidth="1"/>
-    <col min="10" max="10" width="14.109375" style="13" customWidth="1"/>
-    <col min="11" max="16384" width="9.109375" style="13"/>
+    <col min="7" max="7" width="45.140625" style="11" customWidth="1"/>
+    <col min="8" max="8" width="36.28515625" style="15" customWidth="1"/>
+    <col min="9" max="9" width="13.42578125" style="13" customWidth="1"/>
+    <col min="10" max="10" width="14.140625" style="13" customWidth="1"/>
+    <col min="11" max="16384" width="9.140625" style="13"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" s="1" customFormat="1" ht="20.100000000000001" customHeight="1">

</xml_diff>